<commit_message>
Split sector: small digits cleaning
Creation of "residue" parameter to set to 0 small values that can be considered numerical inaccuracies.
Fix in constraint 3 in model_settings.xlsx.
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/Paper example/cvxlab test MARIO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/ops/cvxlab_models/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="206" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DBCD16C-D87A-4522-AF97-5427EF3B0046}"/>
+  <xr:revisionPtr revIDLastSave="265" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4558C336-6794-42EF-A141-7DA09D4C3862}"/>
   <bookViews>
-    <workbookView xWindow="-8920" yWindow="-20500" windowWidth="28800" windowHeight="15370" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="657" activeTab="2" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="5" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="172">
   <si>
     <t>set_key</t>
   </si>
@@ -136,9 +136,6 @@
     <t>Yold</t>
   </si>
   <si>
-    <t>Yold_p</t>
-  </si>
-  <si>
     <t>dim: cols</t>
   </si>
   <si>
@@ -172,9 +169,6 @@
     <t>region_from, region_to, sector_from</t>
   </si>
   <si>
-    <t>dim: rows, filters: {category: [new]}</t>
-  </si>
-  <si>
     <t>region_from, sector_from</t>
   </si>
   <si>
@@ -244,9 +238,6 @@
     <t>category: [stable, parent, new]</t>
   </si>
   <si>
-    <t>I_rs_from_to_n</t>
-  </si>
-  <si>
     <t>dim: cols, filters: {category: [new]}</t>
   </si>
   <si>
@@ -367,18 +358,9 @@
     <t>X</t>
   </si>
   <si>
-    <t>X_pn</t>
-  </si>
-  <si>
-    <t>X_n</t>
-  </si>
-  <si>
     <t>XT</t>
   </si>
   <si>
-    <t>XT_n</t>
-  </si>
-  <si>
     <t>XT_intra</t>
   </si>
   <si>
@@ -391,18 +373,12 @@
     <t>Z_use_n</t>
   </si>
   <si>
-    <t>Z_use_n_to</t>
-  </si>
-  <si>
     <t>Z_use_pn_pn_to</t>
   </si>
   <si>
     <t>Z_use_pn_pn_from</t>
   </si>
   <si>
-    <t>Z_use_pn_pn_imp</t>
-  </si>
-  <si>
     <t>Z_use_st_pn</t>
   </si>
   <si>
@@ -415,9 +391,6 @@
     <t>Z_supply_from</t>
   </si>
   <si>
-    <t>Z_supply_imp</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
@@ -439,9 +412,6 @@
     <t>dim: cols, filters: {category: [parent,new]}</t>
   </si>
   <si>
-    <t>V_n</t>
-  </si>
-  <si>
     <t>factor</t>
   </si>
   <si>
@@ -460,112 +430,130 @@
     <t>V0</t>
   </si>
   <si>
+    <t>Factors of production (rows of V)</t>
+  </si>
+  <si>
+    <t>I_p_r_from_to</t>
+  </si>
+  <si>
+    <t>Constraint 2+: total production of parent and  sectors = total consumption of their outputs</t>
+  </si>
+  <si>
+    <t>Constraint 2-: total production of parent and  sectors = total consumption of their outputs</t>
+  </si>
+  <si>
+    <t>Constraint 3a-: column sum (Avoid redundancy, keep only for )</t>
+  </si>
+  <si>
+    <t>Constraint 3a+: column sum (Avoid redundancy, keep only for )</t>
+  </si>
+  <si>
+    <t>Constraint 4+: trade balance</t>
+  </si>
+  <si>
+    <t>Constraint 4-: trade balance</t>
+  </si>
+  <si>
+    <t>Zold_p_st &lt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Zold_p_st &gt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Z)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Z)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Y)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Y)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Zold_p_p &lt;= (block_diag(I_p_pn,regions) @ Z_use_pn_pn_to @ tran(I_p_pn))*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1b+:  total consumption consistency by region and sector (only parent/ supply) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1b-:  total consumption consistency by region and sector (only parent/ supply) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Zold_p_p &gt;= (block_diag(I_p_pn,regions) @ Z_use_pn_pn_to @ tran(I_p_pn))*(1-eps)</t>
+  </si>
+  <si>
+    <t>Zold_st_p &lt;= ( Z_use_st_pn @ tran(I_p_pn))*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1c+:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1c-:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Zold_st_p &gt;= ( Z_use_st_pn @ tran(I_p_pn))*(1-eps)</t>
+  </si>
+  <si>
+    <t>Z_use_n_pn</t>
+  </si>
+  <si>
+    <t>Z_supply_n</t>
+  </si>
+  <si>
+    <t>Trade &lt;= (mult(Z_supply_n @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_n_pn@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector))*(1+delta)</t>
+  </si>
+  <si>
+    <t>Trade &gt;= (mult(Z_supply_n @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_n_pn@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector))*(1-delta)</t>
+  </si>
+  <si>
+    <t>Yold &lt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Yold &gt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1d+: VA consistency</t>
+  </si>
+  <si>
+    <t>Constraint 1d-: VA consistency</t>
+  </si>
+  <si>
+    <t>Z_use_to</t>
+  </si>
+  <si>
+    <t>V_intra</t>
+  </si>
+  <si>
+    <t>X_intra</t>
+  </si>
+  <si>
+    <t>I_rs_from_to_pn</t>
+  </si>
+  <si>
+    <t>XT_intra &gt;=(I_row_rs @ Z_use_to + I_row_v @ V_intra)*(1-delta)</t>
+  </si>
+  <si>
+    <t>XT_intra &lt;=(I_row_rs @ Z_use_to + I_row_v @ V_intra)*(1+delta)</t>
+  </si>
+  <si>
     <t>Minimize(sum(entropy(Z_use_n,Z0_all_n))+sum(entropy(Z_use_st_p,Z0_st_p))+sum(entropy(V,V0)))</t>
   </si>
   <si>
-    <t>XT_n ==I_rs_from_to_n @ X_n</t>
-  </si>
-  <si>
-    <t>Factors of production (rows of V)</t>
-  </si>
-  <si>
-    <t>I_p_r_from_to</t>
-  </si>
-  <si>
-    <t>Constraint 2+: total production of parent and  sectors = total consumption of their outputs</t>
-  </si>
-  <si>
-    <t>Constraint 2-: total production of parent and  sectors = total consumption of their outputs</t>
-  </si>
-  <si>
-    <t>X_pn&lt;=(Z_supply_from@I_r_st+Z_use_pn_pn_from@I_r_pn+Y_pn_from@I_r_c)*(1+delta)</t>
-  </si>
-  <si>
-    <t>X_pn&gt;=(Z_supply_from@I_r_st+Z_use_pn_pn_from@I_r_pn+Y_pn_from@I_r_c)*(1-delta)</t>
-  </si>
-  <si>
-    <t>XT_intra &gt;=(I_row_rs @ Z_use_n_to + I_row_v @ V_n)*(1-delta)</t>
-  </si>
-  <si>
-    <t>Constraint 3a-: column sum (Avoid redundancy, keep only for )</t>
-  </si>
-  <si>
-    <t>Constraint 3a+: column sum (Avoid redundancy, keep only for )</t>
-  </si>
-  <si>
-    <t>XT_intra &lt;=(I_row_rs @ Z_use_n_to + I_row_v @ V_n)*(1+delta)</t>
-  </si>
-  <si>
-    <t>Trade &gt;= (mult(Z_supply_imp @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_pn_pn_imp@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector))*(1-delta)</t>
-  </si>
-  <si>
-    <t>Trade &lt;= (mult(Z_supply_imp @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_pn_pn_imp@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector))*(1+delta)</t>
-  </si>
-  <si>
-    <t>Constraint 4+: trade balance</t>
-  </si>
-  <si>
-    <t>Constraint 4-: trade balance</t>
-  </si>
-  <si>
-    <t>Vold &gt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1-delta)</t>
-  </si>
-  <si>
-    <t>Vold &lt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1+delta)</t>
-  </si>
-  <si>
-    <t>Constraint 5+: VA consistency</t>
-  </si>
-  <si>
-    <t>Constraint 5-: VA consistency</t>
-  </si>
-  <si>
-    <t>Zold_p_st &lt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1+eps)</t>
-  </si>
-  <si>
-    <t>Zold_p_st &gt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1-eps)</t>
-  </si>
-  <si>
-    <t>Constraint 1a(Z)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1a(Z)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Yold_p &lt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1+eps)</t>
-  </si>
-  <si>
-    <t>Constraint 1a(Y)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1a(Y)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Yold_p &gt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1-eps)</t>
-  </si>
-  <si>
-    <t>Zold_p_p &lt;= (block_diag(I_p_pn,regions) @ Z_use_pn_pn_to @ tran(I_p_pn))*(1+eps)</t>
-  </si>
-  <si>
-    <t>Constraint 1b+:  total consumption consistency by region and sector (only parent/ supply) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1b-:  total consumption consistency by region and sector (only parent/ supply) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Zold_p_p &gt;= (block_diag(I_p_pn,regions) @ Z_use_pn_pn_to @ tran(I_p_pn))*(1-eps)</t>
-  </si>
-  <si>
-    <t>Zold_st_p &lt;= ( Z_use_st_pn @ tran(I_p_pn))*(1+eps)</t>
-  </si>
-  <si>
-    <t>Constraint 1c+:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1c-:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
-  </si>
-  <si>
-    <t>Zold_st_p &gt;= ( Z_use_st_pn @ tran(I_p_pn))*(1-eps)</t>
+    <t>X_intra&lt;=(Z_supply_from@I_r_st+Z_use_pn_pn_from@I_r_pn+Y_pn_from@I_r_c)*(1+delta)</t>
+  </si>
+  <si>
+    <t>X_intra&gt;=(Z_supply_from@I_r_st+Z_use_pn_pn_from@I_r_pn+Y_pn_from@I_r_c)*(1-delta)</t>
+  </si>
+  <si>
+    <t>XT ==I_rs_from_to_pn @ X</t>
+  </si>
+  <si>
+    <t>Vold &lt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1+eps)</t>
+  </si>
+  <si>
+    <t>Vold &gt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1-eps)</t>
   </si>
 </sst>
 </file>
@@ -1015,143 +1003,143 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>140</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>161</v>
+        <v>139</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>163</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C11" t="s">
-        <v>146</v>
+      <c r="C11" s="6" t="s">
+        <v>170</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C12" t="s">
-        <v>147</v>
+      <c r="C12" s="6" t="s">
+        <v>171</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C13" s="7" t="s">
-        <v>151</v>
+      <c r="C13" t="s">
+        <v>167</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C14" s="7" t="s">
-        <v>148</v>
+      <c r="C14" t="s">
+        <v>168</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C15" s="7" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>104</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C16" s="6" t="s">
-        <v>153</v>
+      <c r="C16" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>154</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C17" s="6" t="s">
-        <v>152</v>
+      <c r="C17" s="7" t="s">
+        <v>169</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C18" s="6" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C19" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1195,7 +1183,7 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1206,7 +1194,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -1227,7 +1215,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
         <v>25</v>
@@ -1235,21 +1223,21 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1301,7 +1289,7 @@
         <v>11</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>21</v>
@@ -1316,13 +1304,13 @@
         <v>24</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1336,7 +1324,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -1345,13 +1333,13 @@
         <v>29</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1365,7 +1353,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>30</v>
@@ -1374,13 +1362,13 @@
         <v>29</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1394,22 +1382,22 @@
         <v>15</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J4" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="L4" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1417,370 +1405,376 @@
         <v>31</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>29</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="J10" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="L10" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>109</v>
+        <v>162</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F13" t="s">
-        <v>112</v>
+        <v>106</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="M13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F14" t="s">
-        <v>113</v>
+        <v>107</v>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="M14" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="s">
         <v>39</v>
       </c>
-      <c r="E15" t="s">
-        <v>40</v>
-      </c>
       <c r="F15" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="I15" t="b">
         <v>1</v>
       </c>
       <c r="J15" t="s">
+        <v>53</v>
+      </c>
+      <c r="K15" t="s">
         <v>55</v>
       </c>
-      <c r="K15" t="s">
-        <v>57</v>
-      </c>
       <c r="L15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" t="s">
         <v>39</v>
       </c>
-      <c r="E16" t="s">
-        <v>40</v>
-      </c>
       <c r="F16" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="L16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s">
         <v>39</v>
       </c>
-      <c r="E17" t="s">
-        <v>40</v>
-      </c>
       <c r="F17" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K17" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="L17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18"/>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F18" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="G18"/>
       <c r="H18"/>
@@ -1788,16 +1782,16 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="K18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M18" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="N18"/>
       <c r="O18"/>
@@ -1806,20 +1800,20 @@
     </row>
     <row r="19" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19"/>
       <c r="E19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G19"/>
       <c r="H19"/>
@@ -1827,16 +1821,16 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="K19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L19" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N19"/>
       <c r="O19"/>
@@ -1845,20 +1839,20 @@
     </row>
     <row r="20" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D20"/>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>120</v>
+        <v>152</v>
       </c>
       <c r="G20"/>
       <c r="H20"/>
@@ -1866,16 +1860,16 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N20"/>
       <c r="O20"/>
@@ -1884,20 +1878,20 @@
     </row>
     <row r="21" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D21"/>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F21" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="G21"/>
       <c r="H21"/>
@@ -1905,16 +1899,16 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="K21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M21" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="N21"/>
       <c r="O21"/>
@@ -1923,20 +1917,20 @@
     </row>
     <row r="22" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D22"/>
       <c r="E22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
@@ -1944,16 +1938,16 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K22" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="N22"/>
       <c r="O22"/>
@@ -1962,20 +1956,20 @@
     </row>
     <row r="23" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D23"/>
       <c r="E23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="G23"/>
       <c r="H23"/>
@@ -1983,16 +1977,16 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L23" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N23"/>
       <c r="O23"/>
@@ -2001,52 +1995,52 @@
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" t="s">
         <v>39</v>
       </c>
-      <c r="E24" t="s">
-        <v>40</v>
-      </c>
       <c r="F24" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="I24" t="b">
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" t="s">
         <v>38</v>
-      </c>
-      <c r="C25" t="s">
-        <v>39</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F25" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="G25"/>
       <c r="H25"/>
@@ -2054,17 +2048,17 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K25"/>
       <c r="L25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M25" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="N25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O25"/>
       <c r="P25"/>
@@ -2072,20 +2066,20 @@
     </row>
     <row r="26" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" t="s">
         <v>38</v>
-      </c>
-      <c r="C26" t="s">
-        <v>39</v>
       </c>
       <c r="D26"/>
       <c r="E26" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F26" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="G26"/>
       <c r="H26"/>
@@ -2093,17 +2087,17 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K26"/>
       <c r="L26" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O26"/>
       <c r="P26"/>
@@ -2111,52 +2105,52 @@
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" t="s">
         <v>38</v>
       </c>
-      <c r="C27" t="s">
-        <v>39</v>
-      </c>
       <c r="E27" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F27" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="I27" t="b">
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D28"/>
       <c r="E28" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F28" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="G28"/>
       <c r="H28"/>
@@ -2165,54 +2159,54 @@
       </c>
       <c r="J28"/>
       <c r="K28" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="L28"/>
       <c r="M28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N28"/>
       <c r="O28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P28"/>
       <c r="Q28"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B29" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E29" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F29" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="I29" t="b">
         <v>1</v>
       </c>
       <c r="K29" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="M29" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="O29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>16</v>
@@ -2222,366 +2216,366 @@
         <v>23</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H30" s="8"/>
       <c r="I30" s="8"/>
       <c r="J30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
-        <v>68</v>
+        <v>163</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>68</v>
+        <v>163</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="L31" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M31" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L32" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M32" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L33" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="O34" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K35" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M35" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K36" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M36" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M37" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N37" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L38" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M38" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K39" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L39" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M39" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L40" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M40" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N40" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J41" s="8" t="s">
         <v>29</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L41" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M41" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C42" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L42" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M42" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="43" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K43" s="9" t="s">
         <v>29</v>
@@ -2589,42 +2583,42 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C44" t="s">
         <v>15</v>
       </c>
       <c r="E44" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F44" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="P44" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C45" t="s">
         <v>15</v>
       </c>
       <c r="E45" t="s">
+        <v>89</v>
+      </c>
+      <c r="F45" t="s">
         <v>92</v>
       </c>
-      <c r="F45" t="s">
-        <v>95</v>
-      </c>
       <c r="P45" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2654,8 +2648,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
     <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
     <xsd:element name="properties">
@@ -2704,7 +2698,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2758,8 +2752,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2874,7 +2868,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBE534EA-57E5-4D00-A749-BD6DF04A56B5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BBC26FF-DF30-40C0-960B-B039EC8CD24D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>

</xml_diff>

<commit_message>
Actual implementation of exclusions
When splitting sectors: rom "Exclusions" sheet of the inventory, implement constraint to force values of Z to zero.
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/ops/cvxlab_models/Split_sectors/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/MARIO implementation examples/2r 6s example/impose zeroes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4558C336-6794-42EF-A141-7DA09D4C3862}"/>
+  <xr:revisionPtr revIDLastSave="294" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE71307B-B72F-4365-9712-0A050C224452}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="657" activeTab="2" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
+    <workbookView xWindow="3735" yWindow="-15480" windowWidth="19440" windowHeight="14880" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="5" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="structure_variables" sheetId="7" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="177">
   <si>
     <t>set_key</t>
   </si>
@@ -554,6 +554,21 @@
   </si>
   <si>
     <t>Vold &gt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1-eps)</t>
+  </si>
+  <si>
+    <t>Zero_use_mask</t>
+  </si>
+  <si>
+    <t>Zero_supply_mask</t>
+  </si>
+  <si>
+    <t>ones where prior zeroes</t>
+  </si>
+  <si>
+    <t>0 == mult(Zero_use_mask,Z_use_to)</t>
+  </si>
+  <si>
+    <t>0 == mult(Zero_supply_mask, Z_supply_to)</t>
   </si>
 </sst>
 </file>
@@ -978,7 +993,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E309D5-3CF9-4805-9054-67D3EBAC901C}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -1140,6 +1155,16 @@
       </c>
       <c r="D19" s="5" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C20" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C21" s="7" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1247,7 +1272,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}">
-  <dimension ref="A1:Q45"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" customWidth="1"/>
@@ -1509,10 +1534,10 @@
     </row>
     <row r="9" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>102</v>
+        <v>172</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>60</v>
+        <v>174</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>15</v>
@@ -1521,27 +1546,27 @@
         <v>39</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>103</v>
+        <v>172</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>34</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="L9" s="9" t="s">
         <v>34</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>102</v>
+        <v>173</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>60</v>
+        <v>174</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>15</v>
@@ -1550,181 +1575,175 @@
         <v>39</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>104</v>
+        <v>173</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L10" s="9" t="s">
         <v>34</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>162</v>
+        <v>103</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>66</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>99</v>
+        <v>34</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M12" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F13" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="B14" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J14" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="L12" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" t="s">
-        <v>106</v>
-      </c>
-      <c r="I13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K13" t="s">
-        <v>33</v>
-      </c>
-      <c r="M13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" t="s">
-        <v>62</v>
-      </c>
-      <c r="F14" t="s">
-        <v>107</v>
-      </c>
-      <c r="I14" t="b">
-        <v>1</v>
-      </c>
-      <c r="K14" t="s">
-        <v>123</v>
-      </c>
-      <c r="M14" t="s">
-        <v>99</v>
+      <c r="L14" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C15" t="s">
         <v>38</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I15" t="b">
         <v>1</v>
       </c>
-      <c r="J15" t="s">
-        <v>53</v>
-      </c>
       <c r="K15" t="s">
-        <v>55</v>
-      </c>
-      <c r="L15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C16" t="s">
         <v>38</v>
       </c>
       <c r="E16" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F16" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
-      <c r="J16" t="s">
-        <v>34</v>
-      </c>
       <c r="K16" t="s">
-        <v>66</v>
-      </c>
-      <c r="L16" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="M16" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.35">
@@ -1741,25 +1760,25 @@
         <v>39</v>
       </c>
       <c r="F17" t="s">
-        <v>160</v>
+        <v>109</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="K17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L17" t="s">
         <v>34</v>
       </c>
       <c r="M17" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -1769,36 +1788,29 @@
       <c r="C18" t="s">
         <v>38</v>
       </c>
-      <c r="D18"/>
       <c r="E18" t="s">
         <v>39</v>
       </c>
       <c r="F18" t="s">
-        <v>111</v>
-      </c>
-      <c r="G18"/>
-      <c r="H18"/>
+        <v>110</v>
+      </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="K18" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="L18" t="s">
         <v>34</v>
       </c>
       <c r="M18" t="s">
-        <v>99</v>
-      </c>
-      <c r="N18"/>
-      <c r="O18"/>
-      <c r="P18"/>
-      <c r="Q18"/>
-    </row>
-    <row r="19" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>108</v>
       </c>
@@ -1808,34 +1820,27 @@
       <c r="C19" t="s">
         <v>38</v>
       </c>
-      <c r="D19"/>
       <c r="E19" t="s">
         <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>112</v>
-      </c>
-      <c r="G19"/>
-      <c r="H19"/>
+        <v>160</v>
+      </c>
       <c r="I19" t="b">
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="K19" t="s">
         <v>57</v>
       </c>
       <c r="L19" t="s">
+        <v>34</v>
+      </c>
+      <c r="M19" t="s">
         <v>99</v>
       </c>
-      <c r="M19" t="s">
-        <v>32</v>
-      </c>
-      <c r="N19"/>
-      <c r="O19"/>
-      <c r="P19"/>
-      <c r="Q19"/>
     </row>
     <row r="20" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -1852,7 +1857,7 @@
         <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>152</v>
+        <v>111</v>
       </c>
       <c r="G20"/>
       <c r="H20"/>
@@ -1860,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="K20" t="s">
         <v>57</v>
@@ -1869,7 +1874,7 @@
         <v>34</v>
       </c>
       <c r="M20" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="N20"/>
       <c r="O20"/>
@@ -1891,7 +1896,7 @@
         <v>39</v>
       </c>
       <c r="F21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G21"/>
       <c r="H21"/>
@@ -1899,16 +1904,16 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="K21" t="s">
         <v>57</v>
       </c>
       <c r="L21" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M21" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="N21"/>
       <c r="O21"/>
@@ -1917,10 +1922,10 @@
     </row>
     <row r="22" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
         <v>38</v>
@@ -1930,7 +1935,7 @@
         <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
@@ -1938,16 +1943,16 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L22" t="s">
         <v>34</v>
       </c>
       <c r="M22" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="N22"/>
       <c r="O22"/>
@@ -1956,10 +1961,10 @@
     </row>
     <row r="23" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
         <v>38</v>
@@ -1969,7 +1974,7 @@
         <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G23"/>
       <c r="H23"/>
@@ -1977,23 +1982,23 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="K23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M23" t="s">
         <v>99</v>
-      </c>
-      <c r="M23" t="s">
-        <v>32</v>
       </c>
       <c r="N23"/>
       <c r="O23"/>
       <c r="P23"/>
       <c r="Q23"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>114</v>
       </c>
@@ -2003,17 +2008,20 @@
       <c r="C24" t="s">
         <v>38</v>
       </c>
+      <c r="D24"/>
       <c r="E24" t="s">
         <v>39</v>
       </c>
       <c r="F24" t="s">
-        <v>153</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G24"/>
+      <c r="H24"/>
       <c r="I24" t="b">
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K24" t="s">
         <v>56</v>
@@ -2022,25 +2030,29 @@
         <v>34</v>
       </c>
       <c r="M24" t="s">
-        <v>32</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="Q24"/>
     </row>
     <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C25" t="s">
         <v>38</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F25" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G25"/>
       <c r="H25"/>
@@ -2050,60 +2062,53 @@
       <c r="J25" t="s">
         <v>33</v>
       </c>
-      <c r="K25"/>
+      <c r="K25" t="s">
+        <v>56</v>
+      </c>
       <c r="L25" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M25" t="s">
-        <v>99</v>
-      </c>
-      <c r="N25" t="s">
         <v>32</v>
       </c>
+      <c r="N25"/>
       <c r="O25"/>
       <c r="P25"/>
       <c r="Q25"/>
     </row>
-    <row r="26" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
         <v>38</v>
       </c>
-      <c r="D26"/>
       <c r="E26" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>119</v>
-      </c>
-      <c r="G26"/>
-      <c r="H26"/>
+        <v>153</v>
+      </c>
       <c r="I26" t="b">
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>33</v>
-      </c>
-      <c r="K26"/>
+        <v>35</v>
+      </c>
+      <c r="K26" t="s">
+        <v>56</v>
+      </c>
       <c r="L26" t="s">
-        <v>99</v>
+        <v>34</v>
       </c>
       <c r="M26" t="s">
         <v>32</v>
       </c>
-      <c r="N26" t="s">
-        <v>32</v>
-      </c>
-      <c r="O26"/>
-      <c r="P26"/>
-      <c r="Q26"/>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>117</v>
       </c>
@@ -2113,330 +2118,353 @@
       <c r="C27" t="s">
         <v>38</v>
       </c>
+      <c r="D27"/>
       <c r="E27" t="s">
         <v>68</v>
       </c>
       <c r="F27" t="s">
-        <v>120</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="G27"/>
+      <c r="H27"/>
       <c r="I27" t="b">
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>35</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="K27"/>
       <c r="L27" t="s">
         <v>34</v>
       </c>
       <c r="M27" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="N27" t="s">
         <v>32</v>
       </c>
+      <c r="O27"/>
+      <c r="P27"/>
+      <c r="Q27"/>
     </row>
     <row r="28" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="C28" t="s">
         <v>38</v>
       </c>
       <c r="D28"/>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>68</v>
       </c>
       <c r="F28" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G28"/>
       <c r="H28"/>
       <c r="I28" t="b">
         <v>1</v>
       </c>
-      <c r="J28"/>
-      <c r="K28" t="s">
-        <v>123</v>
-      </c>
-      <c r="L28"/>
+      <c r="J28" t="s">
+        <v>33</v>
+      </c>
+      <c r="K28"/>
+      <c r="L28" t="s">
+        <v>99</v>
+      </c>
       <c r="M28" t="s">
         <v>32</v>
       </c>
-      <c r="N28"/>
-      <c r="O28" t="s">
-        <v>34</v>
-      </c>
+      <c r="N28" t="s">
+        <v>32</v>
+      </c>
+      <c r="O28"/>
       <c r="P28"/>
       <c r="Q28"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="C29" t="s">
         <v>38</v>
       </c>
       <c r="E29" t="s">
-        <v>122</v>
+        <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>161</v>
+        <v>120</v>
       </c>
       <c r="I29" t="b">
         <v>1</v>
       </c>
-      <c r="K29" t="s">
+      <c r="J29" t="s">
+        <v>35</v>
+      </c>
+      <c r="L29" t="s">
+        <v>34</v>
+      </c>
+      <c r="M29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N29" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30"/>
+      <c r="E30" t="s">
+        <v>122</v>
+      </c>
+      <c r="F30" t="s">
+        <v>121</v>
+      </c>
+      <c r="G30"/>
+      <c r="H30"/>
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30"/>
+      <c r="K30" t="s">
         <v>123</v>
       </c>
-      <c r="M29" t="s">
+      <c r="L30"/>
+      <c r="M30" t="s">
+        <v>32</v>
+      </c>
+      <c r="N30"/>
+      <c r="O30" t="s">
+        <v>34</v>
+      </c>
+      <c r="P30"/>
+      <c r="Q30"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" t="s">
+        <v>122</v>
+      </c>
+      <c r="F31" t="s">
+        <v>161</v>
+      </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
+      <c r="K31" t="s">
+        <v>123</v>
+      </c>
+      <c r="M31" t="s">
         <v>99</v>
       </c>
-      <c r="O29" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A30" s="8" t="s">
+      <c r="O31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A32" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B32" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="L30" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="J31" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K31" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="L31" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="M31" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>61</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
       <c r="L32" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="M32" s="8" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
-        <v>127</v>
+        <v>163</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>127</v>
+        <v>163</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>32</v>
+        <v>57</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>76</v>
       </c>
       <c r="L33" s="8" t="s">
         <v>32</v>
       </c>
+      <c r="M33" s="8" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="34" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
-        <v>125</v>
+        <v>51</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>126</v>
+        <v>49</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>125</v>
+        <v>51</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="O34" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L34" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M34" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>78</v>
+        <v>127</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>78</v>
+        <v>127</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="K35" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="M35" s="8" t="s">
-        <v>34</v>
+      <c r="J35" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L35" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>82</v>
+        <v>126</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>62</v>
+        <v>124</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="K36" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="M36" s="8" t="s">
-        <v>34</v>
+      <c r="O36" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>63</v>
       </c>
+      <c r="K37" s="8" t="s">
+        <v>53</v>
+      </c>
       <c r="M37" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="N37" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="L38" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M38" s="8" t="s">
         <v>34</v>
@@ -2444,185 +2472,240 @@
     </row>
     <row r="39" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="K39" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="L39" s="8" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="M39" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N39" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>58</v>
       </c>
+      <c r="K40" s="8" t="s">
+        <v>53</v>
+      </c>
       <c r="L40" s="8" t="s">
         <v>32</v>
       </c>
       <c r="M40" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="N40" s="8" t="s">
-        <v>34</v>
-      </c>
     </row>
     <row r="41" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E41" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L41" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L42" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M42" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N42" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F41" s="8" t="s">
+      <c r="F43" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="G41" s="8" t="s">
+      <c r="G43" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="J41" s="8" t="s">
+      <c r="J43" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K41" s="8" t="s">
+      <c r="K43" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="L41" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="M41" s="8" t="s">
+      <c r="L43" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M43" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="9" t="s">
+    <row r="44" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="B44" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C44" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E44" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F44" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="J42" s="9" t="s">
+      <c r="J44" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="L42" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="M42" s="9" t="s">
+      <c r="L44" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M44" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="43" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="9" t="s">
+    <row r="45" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="B45" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C45" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E45" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="F45" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J43" s="9" t="s">
+      <c r="J45" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K43" s="9" t="s">
+      <c r="K45" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>87</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B46" t="s">
         <v>88</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C46" t="s">
         <v>15</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E46" t="s">
         <v>89</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F46" t="s">
         <v>90</v>
       </c>
-      <c r="P44" t="s">
+      <c r="P46" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>87</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B47" t="s">
         <v>88</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C47" t="s">
         <v>15</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E47" t="s">
         <v>89</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F47" t="s">
         <v>92</v>
       </c>
-      <c r="P45" t="s">
+      <c r="P47" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N30" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
+  <autoFilter ref="A1:N32" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2648,8 +2731,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
     <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
     <xsd:element name="properties">
@@ -2698,7 +2781,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2752,8 +2835,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2868,7 +2951,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BBC26FF-DF30-40C0-960B-B039EC8CD24D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{854781CB-474B-4B47-960A-54F3042E6684}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>

</xml_diff>

<commit_message>
Split routine: zeroes stay zeroes
When parent sector has a null value for a specific transaction, the child corresponding values are imposed for zero. Implemented for Z (along with the exogenously imposed exclusions) and for Y. The exogenously imposed exclusions are not expected for Y at the moment.
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/MARIO implementation examples/2r 6s example/impose zeroes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/MARIO implementation examples/2r 6s example/Y zeroes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="294" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE71307B-B72F-4365-9712-0A050C224452}"/>
+  <xr:revisionPtr revIDLastSave="311" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F49BDC-32D8-4152-85D6-EF6F0778F401}"/>
   <bookViews>
-    <workbookView xWindow="3735" yWindow="-15480" windowWidth="19440" windowHeight="14880" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
+    <workbookView xWindow="-1035" yWindow="-17745" windowWidth="19425" windowHeight="11505" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="5" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="structure_variables" sheetId="7" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="182">
   <si>
     <t>set_key</t>
   </si>
@@ -569,6 +569,21 @@
   </si>
   <si>
     <t>0 == mult(Zero_supply_mask, Z_supply_to)</t>
+  </si>
+  <si>
+    <t>Constraint 5a: impose zeroes</t>
+  </si>
+  <si>
+    <t>Constraint 5c: impose zeroes</t>
+  </si>
+  <si>
+    <t>Constraint 5b: impose zeroes</t>
+  </si>
+  <si>
+    <t>Zero_Y_mask</t>
+  </si>
+  <si>
+    <t>0 == mult(Zero_Y_mask, Y_pn_to)</t>
   </si>
 </sst>
 </file>
@@ -993,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E309D5-3CF9-4805-9054-67D3EBAC901C}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -1161,10 +1176,24 @@
       <c r="C20" s="7" t="s">
         <v>175</v>
       </c>
+      <c r="D20" s="5" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="21" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C21" s="7" t="s">
         <v>176</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C22" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1272,7 +1301,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}">
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" customWidth="1"/>
@@ -1592,34 +1621,34 @@
     </row>
     <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>102</v>
+        <v>180</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>60</v>
+        <v>174</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>103</v>
+        <v>180</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="L11" s="9" t="s">
         <v>34</v>
       </c>
       <c r="M11" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="N11" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>102</v>
       </c>
@@ -1633,13 +1662,13 @@
         <v>39</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="L12" s="9" t="s">
         <v>34</v>
@@ -1650,25 +1679,31 @@
     </row>
     <row r="13" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>162</v>
+        <v>104</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>33</v>
+        <v>53</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>99</v>
+        <v>34</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1685,38 +1720,35 @@
         <v>43</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>105</v>
+        <v>162</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>33</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>106</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" t="s">
-        <v>62</v>
-      </c>
-      <c r="F15" t="s">
-        <v>106</v>
-      </c>
-      <c r="I15" t="b">
-        <v>1</v>
-      </c>
-      <c r="K15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M15" t="s">
+      <c r="L15" s="9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1734,48 +1766,42 @@
         <v>62</v>
       </c>
       <c r="F16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
       <c r="K16" t="s">
-        <v>123</v>
+        <v>33</v>
       </c>
       <c r="M16" t="s">
-        <v>99</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C17" t="s">
         <v>38</v>
       </c>
       <c r="E17" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
-      <c r="J17" t="s">
-        <v>53</v>
-      </c>
       <c r="K17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L17" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="M17" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.35">
@@ -1792,16 +1818,16 @@
         <v>39</v>
       </c>
       <c r="F18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="K18" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="L18" t="s">
         <v>34</v>
@@ -1824,7 +1850,7 @@
         <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>160</v>
+        <v>110</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
@@ -1833,16 +1859,16 @@
         <v>34</v>
       </c>
       <c r="K19" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="L19" t="s">
         <v>34</v>
       </c>
       <c r="M19" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>108</v>
       </c>
@@ -1852,20 +1878,17 @@
       <c r="C20" t="s">
         <v>38</v>
       </c>
-      <c r="D20"/>
       <c r="E20" t="s">
         <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>111</v>
-      </c>
-      <c r="G20"/>
-      <c r="H20"/>
+        <v>160</v>
+      </c>
       <c r="I20" t="b">
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="K20" t="s">
         <v>57</v>
@@ -1876,10 +1899,6 @@
       <c r="M20" t="s">
         <v>99</v>
       </c>
-      <c r="N20"/>
-      <c r="O20"/>
-      <c r="P20"/>
-      <c r="Q20"/>
     </row>
     <row r="21" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1896,7 +1915,7 @@
         <v>39</v>
       </c>
       <c r="F21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G21"/>
       <c r="H21"/>
@@ -1910,10 +1929,10 @@
         <v>57</v>
       </c>
       <c r="L21" t="s">
+        <v>34</v>
+      </c>
+      <c r="M21" t="s">
         <v>99</v>
-      </c>
-      <c r="M21" t="s">
-        <v>32</v>
       </c>
       <c r="N21"/>
       <c r="O21"/>
@@ -1935,7 +1954,7 @@
         <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
@@ -1943,13 +1962,13 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="K22" t="s">
         <v>57</v>
       </c>
       <c r="L22" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M22" t="s">
         <v>32</v>
@@ -1974,7 +1993,7 @@
         <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="G23"/>
       <c r="H23"/>
@@ -1982,7 +2001,7 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="K23" t="s">
         <v>57</v>
@@ -1991,7 +2010,7 @@
         <v>34</v>
       </c>
       <c r="M23" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="N23"/>
       <c r="O23"/>
@@ -2000,10 +2019,10 @@
     </row>
     <row r="24" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C24" t="s">
         <v>38</v>
@@ -2013,7 +2032,7 @@
         <v>39</v>
       </c>
       <c r="F24" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G24"/>
       <c r="H24"/>
@@ -2021,10 +2040,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="K24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L24" t="s">
         <v>34</v>
@@ -2052,7 +2071,7 @@
         <v>39</v>
       </c>
       <c r="F25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G25"/>
       <c r="H25"/>
@@ -2066,17 +2085,17 @@
         <v>56</v>
       </c>
       <c r="L25" t="s">
+        <v>34</v>
+      </c>
+      <c r="M25" t="s">
         <v>99</v>
-      </c>
-      <c r="M25" t="s">
-        <v>32</v>
       </c>
       <c r="N25"/>
       <c r="O25"/>
       <c r="P25"/>
       <c r="Q25"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>114</v>
       </c>
@@ -2086,66 +2105,66 @@
       <c r="C26" t="s">
         <v>38</v>
       </c>
+      <c r="D26"/>
       <c r="E26" t="s">
         <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>153</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G26"/>
+      <c r="H26"/>
       <c r="I26" t="b">
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K26" t="s">
         <v>56</v>
       </c>
       <c r="L26" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M26" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="N26"/>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
         <v>38</v>
       </c>
-      <c r="D27"/>
       <c r="E27" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F27" t="s">
-        <v>118</v>
-      </c>
-      <c r="G27"/>
-      <c r="H27"/>
+        <v>153</v>
+      </c>
       <c r="I27" t="b">
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>33</v>
-      </c>
-      <c r="K27"/>
+        <v>35</v>
+      </c>
+      <c r="K27" t="s">
+        <v>56</v>
+      </c>
       <c r="L27" t="s">
         <v>34</v>
       </c>
       <c r="M27" t="s">
-        <v>99</v>
-      </c>
-      <c r="N27" t="s">
         <v>32</v>
       </c>
-      <c r="O27"/>
-      <c r="P27"/>
-      <c r="Q27"/>
     </row>
     <row r="28" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
@@ -2162,7 +2181,7 @@
         <v>68</v>
       </c>
       <c r="F28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G28"/>
       <c r="H28"/>
@@ -2174,10 +2193,10 @@
       </c>
       <c r="K28"/>
       <c r="L28" t="s">
+        <v>34</v>
+      </c>
+      <c r="M28" t="s">
         <v>99</v>
-      </c>
-      <c r="M28" t="s">
-        <v>32</v>
       </c>
       <c r="N28" t="s">
         <v>32</v>
@@ -2186,7 +2205,7 @@
       <c r="P28"/>
       <c r="Q28"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>117</v>
       </c>
@@ -2196,20 +2215,24 @@
       <c r="C29" t="s">
         <v>38</v>
       </c>
+      <c r="D29"/>
       <c r="E29" t="s">
         <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>120</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="G29"/>
+      <c r="H29"/>
       <c r="I29" t="b">
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>35</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="K29"/>
       <c r="L29" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M29" t="s">
         <v>32</v>
@@ -2217,45 +2240,43 @@
       <c r="N29" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O29"/>
+      <c r="P29"/>
+      <c r="Q29"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="C30" t="s">
         <v>38</v>
       </c>
-      <c r="D30"/>
       <c r="E30" t="s">
-        <v>122</v>
+        <v>68</v>
       </c>
       <c r="F30" t="s">
-        <v>121</v>
-      </c>
-      <c r="G30"/>
-      <c r="H30"/>
+        <v>120</v>
+      </c>
       <c r="I30" t="b">
         <v>1</v>
       </c>
-      <c r="J30"/>
-      <c r="K30" t="s">
-        <v>123</v>
-      </c>
-      <c r="L30"/>
+      <c r="J30" t="s">
+        <v>35</v>
+      </c>
+      <c r="L30" t="s">
+        <v>34</v>
+      </c>
       <c r="M30" t="s">
         <v>32</v>
       </c>
-      <c r="N30"/>
-      <c r="O30" t="s">
-        <v>34</v>
-      </c>
-      <c r="P30"/>
-      <c r="Q30"/>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="N30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>121</v>
       </c>
@@ -2265,87 +2286,92 @@
       <c r="C31" t="s">
         <v>38</v>
       </c>
+      <c r="D31"/>
       <c r="E31" t="s">
         <v>122</v>
       </c>
       <c r="F31" t="s">
-        <v>161</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="G31"/>
+      <c r="H31"/>
       <c r="I31" t="b">
         <v>1</v>
       </c>
+      <c r="J31"/>
       <c r="K31" t="s">
         <v>123</v>
       </c>
+      <c r="L31"/>
       <c r="M31" t="s">
+        <v>32</v>
+      </c>
+      <c r="N31"/>
+      <c r="O31" t="s">
+        <v>34</v>
+      </c>
+      <c r="P31"/>
+      <c r="Q31"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" t="s">
+        <v>38</v>
+      </c>
+      <c r="E32" t="s">
+        <v>122</v>
+      </c>
+      <c r="F32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+      <c r="K32" t="s">
+        <v>123</v>
+      </c>
+      <c r="M32" t="s">
         <v>99</v>
       </c>
-      <c r="O31" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A32" s="8" t="s">
+      <c r="O32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A33" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B33" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
-      <c r="L32" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="D33" s="8"/>
       <c r="E33" s="8" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="J33" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>76</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
       <c r="L33" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="M33" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>49</v>
@@ -2354,102 +2380,108 @@
         <v>16</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="G34" s="8" t="s">
         <v>61</v>
       </c>
+      <c r="J34" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="L34" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M34" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>127</v>
+        <v>51</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>127</v>
+        <v>51</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="J35" s="8" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="L35" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M35" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>124</v>
+        <v>43</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="O36" s="8" t="s">
+      <c r="J36" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L36" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
-        <v>78</v>
+        <v>125</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>79</v>
+        <v>126</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>62</v>
+        <v>124</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>78</v>
+        <v>125</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="K37" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="M37" s="8" t="s">
-        <v>34</v>
+      <c r="O37" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="38" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>16</v>
@@ -2458,13 +2490,13 @@
         <v>62</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>63</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="M38" s="8" t="s">
         <v>34</v>
@@ -2472,62 +2504,59 @@
     </row>
     <row r="39" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>63</v>
       </c>
+      <c r="K39" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="M39" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="N39" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="K40" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="L40" s="8" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="M40" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N40" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B41" s="8" t="s">
         <v>45</v>
@@ -2539,13 +2568,13 @@
         <v>52</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>58</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="L41" s="8" t="s">
         <v>32</v>
@@ -2556,132 +2585,141 @@
     </row>
     <row r="42" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>58</v>
       </c>
+      <c r="K42" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="L42" s="8" t="s">
         <v>32</v>
       </c>
       <c r="M42" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="N42" s="8" t="s">
-        <v>34</v>
-      </c>
     </row>
     <row r="43" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="8" t="s">
-        <v>131</v>
+        <v>83</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L43" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M43" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N43" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F43" s="8" t="s">
+      <c r="F44" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="G43" s="8" t="s">
+      <c r="G44" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="J43" s="8" t="s">
+      <c r="J44" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K43" s="8" t="s">
+      <c r="K44" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="L43" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="M43" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="J44" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="L44" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="M44" s="9" t="s">
+      <c r="L44" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M44" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="45" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C45" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E45" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J45" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L45" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M45" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E46" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F46" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J45" s="9" t="s">
+      <c r="J46" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K45" s="9" t="s">
+      <c r="K46" s="9" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>87</v>
-      </c>
-      <c r="B46" t="s">
-        <v>88</v>
-      </c>
-      <c r="C46" t="s">
-        <v>15</v>
-      </c>
-      <c r="E46" t="s">
-        <v>89</v>
-      </c>
-      <c r="F46" t="s">
-        <v>90</v>
-      </c>
-      <c r="P46" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.35">
@@ -2698,14 +2736,34 @@
         <v>89</v>
       </c>
       <c r="F47" t="s">
+        <v>90</v>
+      </c>
+      <c r="P47" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" t="s">
+        <v>88</v>
+      </c>
+      <c r="C48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48" t="s">
+        <v>89</v>
+      </c>
+      <c r="F48" t="s">
         <v>92</v>
       </c>
-      <c r="P47" t="s">
+      <c r="P48" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N32" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
+  <autoFilter ref="A1:N33" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2951,7 +3009,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{854781CB-474B-4B47-960A-54F3042E6684}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CC58319-9FA4-48F4-98E3-7FCDE2D926A2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>

</xml_diff>

<commit_message>
Zero mask on V as well
Added constraint so that zeroes stay zeroes in V as well
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/MARIO implementation examples/2r 6s example/Y zeroes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/Paper example/more precise/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="311" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F49BDC-32D8-4152-85D6-EF6F0778F401}"/>
+  <xr:revisionPtr revIDLastSave="321" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B485BE8-7AE4-4E82-B0AB-453687E4AC2A}"/>
   <bookViews>
-    <workbookView xWindow="-1035" yWindow="-17745" windowWidth="19425" windowHeight="11505" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="5" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="structure_variables" sheetId="7" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="185">
   <si>
     <t>set_key</t>
   </si>
@@ -584,6 +584,15 @@
   </si>
   <si>
     <t>0 == mult(Zero_Y_mask, Y_pn_to)</t>
+  </si>
+  <si>
+    <t>Constraint 5d: impose zeroes</t>
+  </si>
+  <si>
+    <t>Zero_V_mask</t>
+  </si>
+  <si>
+    <t>0 == mult(Zero_V_mask, V)</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E309D5-3CF9-4805-9054-67D3EBAC901C}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -1194,6 +1203,14 @@
       </c>
       <c r="D22" s="5" t="s">
         <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C23" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -1301,7 +1318,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}">
-  <dimension ref="A1:Q48"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" customWidth="1"/>
@@ -1648,36 +1665,33 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>102</v>
+        <v>183</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>60</v>
+        <v>174</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>39</v>
+        <v>122</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>34</v>
+        <v>183</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O12" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>102</v>
       </c>
@@ -1691,13 +1705,13 @@
         <v>39</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>34</v>
@@ -1708,25 +1722,31 @@
     </row>
     <row r="14" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>162</v>
+        <v>104</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>33</v>
+        <v>53</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>99</v>
+        <v>34</v>
+      </c>
+      <c r="M14" s="9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1743,38 +1763,35 @@
         <v>43</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>105</v>
+        <v>162</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>106</v>
-      </c>
-      <c r="B16" t="s">
-        <v>100</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" t="s">
-        <v>62</v>
-      </c>
-      <c r="F16" t="s">
-        <v>106</v>
-      </c>
-      <c r="I16" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M16" t="s">
+      <c r="L16" s="9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1792,48 +1809,42 @@
         <v>62</v>
       </c>
       <c r="F17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="K17" t="s">
-        <v>123</v>
+        <v>33</v>
       </c>
       <c r="M17" t="s">
-        <v>99</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
         <v>38</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F18" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
-      <c r="J18" t="s">
-        <v>53</v>
-      </c>
       <c r="K18" t="s">
-        <v>55</v>
-      </c>
-      <c r="L18" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="M18" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.35">
@@ -1850,16 +1861,16 @@
         <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="K19" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="L19" t="s">
         <v>34</v>
@@ -1882,7 +1893,7 @@
         <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>160</v>
+        <v>110</v>
       </c>
       <c r="I20" t="b">
         <v>1</v>
@@ -1891,16 +1902,16 @@
         <v>34</v>
       </c>
       <c r="K20" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="L20" t="s">
         <v>34</v>
       </c>
       <c r="M20" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>108</v>
       </c>
@@ -1910,20 +1921,17 @@
       <c r="C21" t="s">
         <v>38</v>
       </c>
-      <c r="D21"/>
       <c r="E21" t="s">
         <v>39</v>
       </c>
       <c r="F21" t="s">
-        <v>111</v>
-      </c>
-      <c r="G21"/>
-      <c r="H21"/>
+        <v>160</v>
+      </c>
       <c r="I21" t="b">
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="K21" t="s">
         <v>57</v>
@@ -1934,10 +1942,6 @@
       <c r="M21" t="s">
         <v>99</v>
       </c>
-      <c r="N21"/>
-      <c r="O21"/>
-      <c r="P21"/>
-      <c r="Q21"/>
     </row>
     <row r="22" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -1954,7 +1958,7 @@
         <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
@@ -1968,10 +1972,10 @@
         <v>57</v>
       </c>
       <c r="L22" t="s">
+        <v>34</v>
+      </c>
+      <c r="M22" t="s">
         <v>99</v>
-      </c>
-      <c r="M22" t="s">
-        <v>32</v>
       </c>
       <c r="N22"/>
       <c r="O22"/>
@@ -1993,7 +1997,7 @@
         <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
       <c r="G23"/>
       <c r="H23"/>
@@ -2001,13 +2005,13 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="K23" t="s">
         <v>57</v>
       </c>
       <c r="L23" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M23" t="s">
         <v>32</v>
@@ -2032,7 +2036,7 @@
         <v>39</v>
       </c>
       <c r="F24" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="G24"/>
       <c r="H24"/>
@@ -2040,7 +2044,7 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="K24" t="s">
         <v>57</v>
@@ -2049,7 +2053,7 @@
         <v>34</v>
       </c>
       <c r="M24" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="N24"/>
       <c r="O24"/>
@@ -2058,10 +2062,10 @@
     </row>
     <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
         <v>38</v>
@@ -2071,7 +2075,7 @@
         <v>39</v>
       </c>
       <c r="F25" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G25"/>
       <c r="H25"/>
@@ -2079,10 +2083,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="K25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L25" t="s">
         <v>34</v>
@@ -2110,7 +2114,7 @@
         <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G26"/>
       <c r="H26"/>
@@ -2124,17 +2128,17 @@
         <v>56</v>
       </c>
       <c r="L26" t="s">
+        <v>34</v>
+      </c>
+      <c r="M26" t="s">
         <v>99</v>
-      </c>
-      <c r="M26" t="s">
-        <v>32</v>
       </c>
       <c r="N26"/>
       <c r="O26"/>
       <c r="P26"/>
       <c r="Q26"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>114</v>
       </c>
@@ -2144,66 +2148,66 @@
       <c r="C27" t="s">
         <v>38</v>
       </c>
+      <c r="D27"/>
       <c r="E27" t="s">
         <v>39</v>
       </c>
       <c r="F27" t="s">
-        <v>153</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G27"/>
+      <c r="H27"/>
       <c r="I27" t="b">
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K27" t="s">
         <v>56</v>
       </c>
       <c r="L27" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M27" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="N27"/>
+      <c r="O27"/>
+      <c r="P27"/>
+      <c r="Q27"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C28" t="s">
         <v>38</v>
       </c>
-      <c r="D28"/>
       <c r="E28" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F28" t="s">
-        <v>118</v>
-      </c>
-      <c r="G28"/>
-      <c r="H28"/>
+        <v>153</v>
+      </c>
       <c r="I28" t="b">
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>33</v>
-      </c>
-      <c r="K28"/>
+        <v>35</v>
+      </c>
+      <c r="K28" t="s">
+        <v>56</v>
+      </c>
       <c r="L28" t="s">
         <v>34</v>
       </c>
       <c r="M28" t="s">
-        <v>99</v>
-      </c>
-      <c r="N28" t="s">
         <v>32</v>
       </c>
-      <c r="O28"/>
-      <c r="P28"/>
-      <c r="Q28"/>
     </row>
     <row r="29" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
@@ -2220,7 +2224,7 @@
         <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G29"/>
       <c r="H29"/>
@@ -2232,10 +2236,10 @@
       </c>
       <c r="K29"/>
       <c r="L29" t="s">
+        <v>34</v>
+      </c>
+      <c r="M29" t="s">
         <v>99</v>
-      </c>
-      <c r="M29" t="s">
-        <v>32</v>
       </c>
       <c r="N29" t="s">
         <v>32</v>
@@ -2244,7 +2248,7 @@
       <c r="P29"/>
       <c r="Q29"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>117</v>
       </c>
@@ -2254,20 +2258,24 @@
       <c r="C30" t="s">
         <v>38</v>
       </c>
+      <c r="D30"/>
       <c r="E30" t="s">
         <v>68</v>
       </c>
       <c r="F30" t="s">
-        <v>120</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="G30"/>
+      <c r="H30"/>
       <c r="I30" t="b">
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>35</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="K30"/>
       <c r="L30" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="M30" t="s">
         <v>32</v>
@@ -2275,45 +2283,43 @@
       <c r="N30" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O30"/>
+      <c r="P30"/>
+      <c r="Q30"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="C31" t="s">
         <v>38</v>
       </c>
-      <c r="D31"/>
       <c r="E31" t="s">
-        <v>122</v>
+        <v>68</v>
       </c>
       <c r="F31" t="s">
-        <v>121</v>
-      </c>
-      <c r="G31"/>
-      <c r="H31"/>
+        <v>120</v>
+      </c>
       <c r="I31" t="b">
         <v>1</v>
       </c>
-      <c r="J31"/>
-      <c r="K31" t="s">
-        <v>123</v>
-      </c>
-      <c r="L31"/>
+      <c r="J31" t="s">
+        <v>35</v>
+      </c>
+      <c r="L31" t="s">
+        <v>34</v>
+      </c>
       <c r="M31" t="s">
         <v>32</v>
       </c>
-      <c r="N31"/>
-      <c r="O31" t="s">
-        <v>34</v>
-      </c>
-      <c r="P31"/>
-      <c r="Q31"/>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="N31" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>121</v>
       </c>
@@ -2323,87 +2329,92 @@
       <c r="C32" t="s">
         <v>38</v>
       </c>
+      <c r="D32"/>
       <c r="E32" t="s">
         <v>122</v>
       </c>
       <c r="F32" t="s">
-        <v>161</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="G32"/>
+      <c r="H32"/>
       <c r="I32" t="b">
         <v>1</v>
       </c>
+      <c r="J32"/>
       <c r="K32" t="s">
         <v>123</v>
       </c>
+      <c r="L32"/>
       <c r="M32" t="s">
+        <v>32</v>
+      </c>
+      <c r="N32"/>
+      <c r="O32" t="s">
+        <v>34</v>
+      </c>
+      <c r="P32"/>
+      <c r="Q32"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" t="s">
+        <v>38</v>
+      </c>
+      <c r="E33" t="s">
+        <v>122</v>
+      </c>
+      <c r="F33" t="s">
+        <v>161</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K33" t="s">
+        <v>123</v>
+      </c>
+      <c r="M33" t="s">
         <v>99</v>
       </c>
-      <c r="O32" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
+      <c r="O33" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A34" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B34" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
-      <c r="L33" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="J34" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K34" s="8" t="s">
-        <v>76</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
       <c r="L34" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="M34" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="B35" s="8" t="s">
         <v>49</v>
@@ -2412,102 +2423,108 @@
         <v>16</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>61</v>
       </c>
+      <c r="J35" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="L35" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M35" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
-        <v>127</v>
+        <v>51</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>127</v>
+        <v>51</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="J36" s="8" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="L36" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M36" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>124</v>
+        <v>43</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="O37" s="8" t="s">
+      <c r="J37" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L37" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="38" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>78</v>
+        <v>125</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>79</v>
+        <v>126</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>62</v>
+        <v>124</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>78</v>
+        <v>125</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="K38" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="M38" s="8" t="s">
-        <v>34</v>
+      <c r="O38" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>16</v>
@@ -2516,13 +2533,13 @@
         <v>62</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>63</v>
       </c>
       <c r="K39" s="8" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="M39" s="8" t="s">
         <v>34</v>
@@ -2530,62 +2547,59 @@
     </row>
     <row r="40" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>63</v>
       </c>
+      <c r="K40" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="M40" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="N40" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="K41" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="L41" s="8" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="M41" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N41" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="42" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>45</v>
@@ -2597,13 +2611,13 @@
         <v>52</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>58</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="L42" s="8" t="s">
         <v>32</v>
@@ -2614,132 +2628,141 @@
     </row>
     <row r="43" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="8" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="G43" s="8" t="s">
         <v>58</v>
       </c>
+      <c r="K43" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="L43" s="8" t="s">
         <v>32</v>
       </c>
       <c r="M43" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="N43" s="8" t="s">
-        <v>34</v>
-      </c>
     </row>
     <row r="44" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
-        <v>131</v>
+        <v>83</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E44" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L44" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M44" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N44" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E45" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F44" s="8" t="s">
+      <c r="F45" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="G44" s="8" t="s">
+      <c r="G45" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="J44" s="8" t="s">
+      <c r="J45" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K44" s="8" t="s">
+      <c r="K45" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="L44" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="M44" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B45" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="J45" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="L45" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="M45" s="9" t="s">
+      <c r="L45" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M45" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E46" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J46" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L46" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M46" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F47" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J46" s="9" t="s">
+      <c r="J47" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K46" s="9" t="s">
+      <c r="K47" s="9" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>87</v>
-      </c>
-      <c r="B47" t="s">
-        <v>88</v>
-      </c>
-      <c r="C47" t="s">
-        <v>15</v>
-      </c>
-      <c r="E47" t="s">
-        <v>89</v>
-      </c>
-      <c r="F47" t="s">
-        <v>90</v>
-      </c>
-      <c r="P47" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.35">
@@ -2756,41 +2779,41 @@
         <v>89</v>
       </c>
       <c r="F48" t="s">
+        <v>90</v>
+      </c>
+      <c r="P48" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" t="s">
+        <v>88</v>
+      </c>
+      <c r="C49" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49" t="s">
+        <v>89</v>
+      </c>
+      <c r="F49" t="s">
         <v>92</v>
       </c>
-      <c r="P48" t="s">
+      <c r="P49" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N33" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
+  <autoFilter ref="A1:N34" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
     <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
     <xsd:element name="properties">
@@ -2839,7 +2862,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2893,8 +2916,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2983,10 +3006,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91788BB2-4A3F-4B3D-BB9A-4A497CBAE5D7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A9A8DFA-706C-482B-B3AD-CDE1EC1BA204}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3009,20 +3063,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CC58319-9FA4-48F4-98E3-7FCDE2D926A2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91788BB2-4A3F-4B3D-BB9A-4A497CBAE5D7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
-    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>